<commit_message>
speed experiment real run
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios122.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios122.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,27 +429,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>scenario_index</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>
@@ -461,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>28725.35614758425</v>
+        <v>26949.12095686317</v>
       </c>
     </row>
     <row r="3">
@@ -524,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>23963.01774121611</v>
+        <v>30863.67153832983</v>
       </c>
     </row>
     <row r="6">
@@ -587,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>14928.8320178776</v>
+        <v>7861.434834207193</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>29138.17913844815</v>
+        <v>12077.26032149434</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>7284.544784612039</v>
+        <v>3019.315080373586</v>
       </c>
     </row>
     <row r="14">
@@ -713,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>46487.69937914996</v>
+        <v>57829.12348425346</v>
       </c>
     </row>
     <row r="15">
@@ -776,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11621.98641144057</v>
+        <v>13613.69252462445</v>
       </c>
     </row>
     <row r="18">
@@ -839,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>36844.09611630544</v>
+        <v>26878.69637759407</v>
       </c>
     </row>
     <row r="21">
@@ -902,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>30755.76046864681</v>
+        <v>27598.36157122732</v>
       </c>
     </row>
     <row r="24">
@@ -965,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>10739.47105274393</v>
+        <v>9949.90729408066</v>
       </c>
     </row>
     <row r="27">
@@ -1028,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>23255.36026151579</v>
+        <v>21393.52218296603</v>
       </c>
     </row>
     <row r="30">
@@ -1070,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5813.840065378947</v>
+        <v>5348.380545741506</v>
       </c>
     </row>
     <row r="32">
@@ -1091,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>43048.73460781306</v>
+        <v>54396.08709948022</v>
       </c>
     </row>
     <row r="33">
@@ -1154,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>10753.51342411154</v>
+        <v>9821.18218240112</v>
       </c>
     </row>
     <row r="36">

</xml_diff>

<commit_message>
speed experiment half success
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios122.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios122.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,27 +417,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>scenario_index</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>

</xml_diff>

<commit_message>
Updated speed experiment to be consistent with experiment parameters
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios122.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios122.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,27 +429,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>scenario_index</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>
@@ -461,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>26949.12095686317</v>
+        <v>28725.35614758425</v>
       </c>
     </row>
     <row r="3">
@@ -524,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>30863.67153832983</v>
+        <v>23963.01774121611</v>
       </c>
     </row>
     <row r="6">
@@ -587,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>7861.434834207193</v>
+        <v>14928.8320178776</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>12077.26032149434</v>
+        <v>29138.17913844815</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3019.315080373586</v>
+        <v>7284.544784612039</v>
       </c>
     </row>
     <row r="14">
@@ -713,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>57829.12348425346</v>
+        <v>46487.69937914996</v>
       </c>
     </row>
     <row r="15">
@@ -776,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>13613.69252462445</v>
+        <v>11621.98641144057</v>
       </c>
     </row>
     <row r="18">
@@ -839,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>26878.69637759407</v>
+        <v>36844.09611630544</v>
       </c>
     </row>
     <row r="21">
@@ -902,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>27598.36157122732</v>
+        <v>30755.76046864681</v>
       </c>
     </row>
     <row r="24">
@@ -965,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>9949.90729408066</v>
+        <v>10739.47105274393</v>
       </c>
     </row>
     <row r="27">
@@ -1028,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>21393.52218296603</v>
+        <v>23255.36026151579</v>
       </c>
     </row>
     <row r="30">
@@ -1070,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5348.380545741506</v>
+        <v>5813.840065378947</v>
       </c>
     </row>
     <row r="32">
@@ -1091,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>54396.08709948022</v>
+        <v>43048.73460781306</v>
       </c>
     </row>
     <row r="33">
@@ -1154,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>9821.18218240112</v>
+        <v>10753.51342411154</v>
       </c>
     </row>
     <row r="36">

</xml_diff>